<commit_message>
Added new student records
</commit_message>
<xml_diff>
--- a/excel/II DS&AI.xlsx
+++ b/excel/II DS&AI.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\DS AI\ACADEMIA 2025-2026\Even sem 2025-2026\ROLL CALL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saket\Desktop\Jr Tech\Technical skills\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58172A38-D2EE-4EA3-8E9F-3E9667083F73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25E6B600-1E58-4D5F-A258-12EF85229393}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DS(AI)-AA" sheetId="1" r:id="rId1"/>
@@ -24,12 +24,12 @@
     <definedName name="_xlnm.Print_Area" localSheetId="2">'DS(AI)-BA'!$A$2:$E$41</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'DS(AI)-BB'!$A$2:$E$40</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="237">
   <si>
     <t>ROLL CALL - EVEN SEMESTER 2025-2026 - II YEAR / IV SEM 
 (2024-2028 BATCH - SHIFT I)</t>
@@ -766,6 +766,9 @@
   </si>
   <si>
     <t>11.05.26</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -959,7 +962,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1081,24 +1084,6 @@
     <xf numFmtId="0" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1112,10 +1097,55 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="10" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2964,35 +2994,37 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F201"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.42578125" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="46.7109375" customWidth="1"/>
+    <col min="1" max="1" width="6.42578125" style="50" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="7" style="50" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.42578125" style="50" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20" style="50" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="46.7109375" style="50" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="50"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="52"/>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
-    </row>
-    <row r="2" spans="1:5" s="24" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="23"/>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23" t="s">
+    <row r="1" spans="1:8" ht="66" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="49"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="H1"/>
+    </row>
+    <row r="2" spans="1:8" s="52" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="51"/>
+      <c r="B2" s="51"/>
+      <c r="C2" s="51" t="s">
         <v>207</v>
       </c>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23" t="s">
+      <c r="D2" s="51"/>
+      <c r="E2" s="51" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="53" t="s">
         <v>0</v>
       </c>
@@ -3001,14 +3033,14 @@
       <c r="D3" s="53"/>
       <c r="E3" s="53"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>3</v>
       </c>
       <c r="D4" s="3" t="s">
@@ -3018,14 +3050,14 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="5">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="54">
         <v>2024</v>
       </c>
       <c r="B5" s="4">
         <v>1</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D5" s="6">
@@ -3035,15 +3067,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="5">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="54">
         <v>2024</v>
       </c>
       <c r="B6" s="4">
         <f t="shared" ref="B6:B65" si="0">B5+1</f>
         <v>2</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D6" s="6">
@@ -3053,15 +3085,15 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="5">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="54">
         <v>2024</v>
       </c>
       <c r="B7" s="4">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D7" s="6">
@@ -3071,15 +3103,15 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="5">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="54">
         <v>2024</v>
       </c>
       <c r="B8" s="4">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D8" s="6">
@@ -3089,15 +3121,15 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="5">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="54">
         <v>2024</v>
       </c>
       <c r="B9" s="4">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D9" s="6">
@@ -3107,15 +3139,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="5">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="54">
         <v>2024</v>
       </c>
       <c r="B10" s="4">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D10" s="6">
@@ -3125,15 +3157,15 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="5">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="54">
         <v>2024</v>
       </c>
       <c r="B11" s="4">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D11" s="6">
@@ -3143,15 +3175,15 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="5">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="54">
         <v>2024</v>
       </c>
       <c r="B12" s="4">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D12" s="6">
@@ -3161,15 +3193,15 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="5">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="54">
         <v>2024</v>
       </c>
       <c r="B13" s="4">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D13" s="6">
@@ -3179,15 +3211,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="5">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="54">
         <v>2024</v>
       </c>
       <c r="B14" s="4">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D14" s="6">
@@ -3197,15 +3229,15 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="5">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="54">
         <v>2024</v>
       </c>
       <c r="B15" s="4">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D15" s="6">
@@ -3215,15 +3247,15 @@
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="5">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="54">
         <v>2024</v>
       </c>
       <c r="B16" s="4">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D16" s="6">
@@ -3234,14 +3266,14 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="5">
+      <c r="A17" s="54">
         <v>2024</v>
       </c>
       <c r="B17" s="4">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D17" s="6">
@@ -3252,14 +3284,14 @@
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="5">
+      <c r="A18" s="54">
         <v>2024</v>
       </c>
       <c r="B18" s="4">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D18" s="6">
@@ -3270,14 +3302,14 @@
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="5">
+      <c r="A19" s="54">
         <v>2024</v>
       </c>
       <c r="B19" s="4">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D19" s="6">
@@ -3288,14 +3320,14 @@
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="5">
+      <c r="A20" s="54">
         <v>2024</v>
       </c>
       <c r="B20" s="4">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D20" s="6">
@@ -3306,14 +3338,14 @@
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="5">
+      <c r="A21" s="54">
         <v>2024</v>
       </c>
       <c r="B21" s="4">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D21" s="6">
@@ -3324,14 +3356,14 @@
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="5">
+      <c r="A22" s="54">
         <v>2024</v>
       </c>
       <c r="B22" s="4">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C22" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D22" s="6">
@@ -3342,14 +3374,14 @@
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="5">
+      <c r="A23" s="54">
         <v>2024</v>
       </c>
       <c r="B23" s="4">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D23" s="6">
@@ -3360,14 +3392,14 @@
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="5">
+      <c r="A24" s="54">
         <v>2024</v>
       </c>
       <c r="B24" s="4">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="C24" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D24" s="6">
@@ -3378,14 +3410,14 @@
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="5">
+      <c r="A25" s="54">
         <v>2024</v>
       </c>
       <c r="B25" s="4">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C25" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D25" s="6">
@@ -3396,14 +3428,14 @@
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="5">
+      <c r="A26" s="54">
         <v>2024</v>
       </c>
       <c r="B26" s="4">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D26" s="6">
@@ -3414,14 +3446,14 @@
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="5">
+      <c r="A27" s="54">
         <v>2024</v>
       </c>
       <c r="B27" s="4">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C27" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D27" s="6">
@@ -3432,14 +3464,14 @@
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="5">
+      <c r="A28" s="54">
         <v>2024</v>
       </c>
       <c r="B28" s="4">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C28" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D28" s="6">
@@ -3450,14 +3482,14 @@
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="5">
+      <c r="A29" s="54">
         <v>2024</v>
       </c>
       <c r="B29" s="4">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="C29" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D29" s="6">
@@ -3468,14 +3500,14 @@
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="5">
+      <c r="A30" s="54">
         <v>2024</v>
       </c>
       <c r="B30" s="4">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="C30" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D30" s="6">
@@ -3486,14 +3518,14 @@
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="5">
+      <c r="A31" s="54">
         <v>2024</v>
       </c>
       <c r="B31" s="4">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="C31" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D31" s="6">
@@ -3504,14 +3536,14 @@
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="5">
+      <c r="A32" s="54">
         <v>2024</v>
       </c>
       <c r="B32" s="4">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="C32" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D32" s="6">
@@ -3522,14 +3554,14 @@
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="5">
+      <c r="A33" s="54">
         <v>2024</v>
       </c>
       <c r="B33" s="4">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="C33" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D33" s="6">
@@ -3540,14 +3572,14 @@
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="5">
+      <c r="A34" s="54">
         <v>2024</v>
       </c>
       <c r="B34" s="4">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="C34" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D34" s="6">
@@ -3558,14 +3590,14 @@
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="5">
+      <c r="A35" s="54">
         <v>2024</v>
       </c>
       <c r="B35" s="4">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="C35" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D35" s="6">
@@ -3576,14 +3608,14 @@
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="5">
+      <c r="A36" s="54">
         <v>2024</v>
       </c>
       <c r="B36" s="4">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="C36" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D36" s="6">
@@ -3594,14 +3626,14 @@
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="5">
+      <c r="A37" s="54">
         <v>2024</v>
       </c>
       <c r="B37" s="4">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="C37" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D37" s="6">
@@ -3612,14 +3644,14 @@
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="5">
+      <c r="A38" s="54">
         <v>2024</v>
       </c>
       <c r="B38" s="4">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="C38" s="1" t="s">
+      <c r="C38" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D38" s="6">
@@ -3630,14 +3662,14 @@
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="5">
+      <c r="A39" s="54">
         <v>2024</v>
       </c>
       <c r="B39" s="4">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="C39" s="1" t="s">
+      <c r="C39" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D39" s="6">
@@ -3648,14 +3680,14 @@
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="5">
+      <c r="A40" s="54">
         <v>2024</v>
       </c>
       <c r="B40" s="4">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="C40" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D40" s="6">
@@ -3666,14 +3698,14 @@
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="5">
+      <c r="A41" s="54">
         <v>2024</v>
       </c>
       <c r="B41" s="4">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="C41" s="1" t="s">
+      <c r="C41" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D41" s="6">
@@ -3684,14 +3716,14 @@
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="5">
+      <c r="A42" s="54">
         <v>2024</v>
       </c>
       <c r="B42" s="4">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="C42" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D42" s="6">
@@ -3702,14 +3734,14 @@
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="5">
+      <c r="A43" s="54">
         <v>2024</v>
       </c>
       <c r="B43" s="4">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
-      <c r="C43" s="1" t="s">
+      <c r="C43" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D43" s="6">
@@ -3720,14 +3752,14 @@
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="5">
+      <c r="A44" s="54">
         <v>2024</v>
       </c>
       <c r="B44" s="4">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="C44" s="1" t="s">
+      <c r="C44" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D44" s="6">
@@ -3738,14 +3770,14 @@
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" s="5">
+      <c r="A45" s="54">
         <v>2024</v>
       </c>
       <c r="B45" s="4">
         <f t="shared" si="0"/>
         <v>41</v>
       </c>
-      <c r="C45" s="1" t="s">
+      <c r="C45" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D45" s="6">
@@ -3756,14 +3788,14 @@
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="5">
+      <c r="A46" s="54">
         <v>2024</v>
       </c>
       <c r="B46" s="4">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="C46" s="1" t="s">
+      <c r="C46" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D46" s="6">
@@ -3774,14 +3806,14 @@
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" s="5">
+      <c r="A47" s="54">
         <v>2024</v>
       </c>
       <c r="B47" s="4">
         <f t="shared" si="0"/>
         <v>43</v>
       </c>
-      <c r="C47" s="1" t="s">
+      <c r="C47" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D47" s="6">
@@ -3792,14 +3824,14 @@
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="5">
+      <c r="A48" s="54">
         <v>2024</v>
       </c>
       <c r="B48" s="4">
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
-      <c r="C48" s="1" t="s">
+      <c r="C48" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D48" s="6">
@@ -3810,14 +3842,14 @@
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" s="5">
+      <c r="A49" s="54">
         <v>2024</v>
       </c>
       <c r="B49" s="4">
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
-      <c r="C49" s="1" t="s">
+      <c r="C49" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D49" s="6">
@@ -3828,14 +3860,14 @@
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="5">
+      <c r="A50" s="54">
         <v>2024</v>
       </c>
       <c r="B50" s="4">
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
-      <c r="C50" s="1" t="s">
+      <c r="C50" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D50" s="6">
@@ -3846,14 +3878,14 @@
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="5">
+      <c r="A51" s="54">
         <v>2024</v>
       </c>
       <c r="B51" s="4">
         <f t="shared" si="0"/>
         <v>47</v>
       </c>
-      <c r="C51" s="1" t="s">
+      <c r="C51" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D51" s="6">
@@ -3864,14 +3896,14 @@
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="5">
+      <c r="A52" s="54">
         <v>2024</v>
       </c>
       <c r="B52" s="4">
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
-      <c r="C52" s="1" t="s">
+      <c r="C52" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D52" s="6">
@@ -3882,14 +3914,14 @@
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="5">
+      <c r="A53" s="54">
         <v>2024</v>
       </c>
       <c r="B53" s="4">
         <f t="shared" si="0"/>
         <v>49</v>
       </c>
-      <c r="C53" s="1" t="s">
+      <c r="C53" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D53" s="6">
@@ -3900,14 +3932,14 @@
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="5">
+      <c r="A54" s="54">
         <v>2024</v>
       </c>
       <c r="B54" s="4">
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
-      <c r="C54" s="1" t="s">
+      <c r="C54" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D54" s="6">
@@ -3918,14 +3950,14 @@
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" s="5">
+      <c r="A55" s="54">
         <v>2024</v>
       </c>
       <c r="B55" s="4">
         <f t="shared" si="0"/>
         <v>51</v>
       </c>
-      <c r="C55" s="1" t="s">
+      <c r="C55" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D55" s="6">
@@ -3936,14 +3968,14 @@
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" s="5">
+      <c r="A56" s="54">
         <v>2024</v>
       </c>
       <c r="B56" s="4">
         <f t="shared" si="0"/>
         <v>52</v>
       </c>
-      <c r="C56" s="1" t="s">
+      <c r="C56" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D56" s="6">
@@ -3954,14 +3986,14 @@
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="5">
+      <c r="A57" s="54">
         <v>2024</v>
       </c>
       <c r="B57" s="4">
         <f t="shared" si="0"/>
         <v>53</v>
       </c>
-      <c r="C57" s="1" t="s">
+      <c r="C57" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D57" s="6">
@@ -3972,14 +4004,14 @@
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" s="5">
+      <c r="A58" s="54">
         <v>2024</v>
       </c>
       <c r="B58" s="4">
         <f t="shared" si="0"/>
         <v>54</v>
       </c>
-      <c r="C58" s="1" t="s">
+      <c r="C58" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D58" s="6">
@@ -3990,14 +4022,14 @@
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" s="5">
+      <c r="A59" s="54">
         <v>2024</v>
       </c>
       <c r="B59" s="4">
         <f t="shared" si="0"/>
         <v>55</v>
       </c>
-      <c r="C59" s="1" t="s">
+      <c r="C59" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D59" s="6">
@@ -4008,14 +4040,14 @@
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" s="5">
+      <c r="A60" s="54">
         <v>2024</v>
       </c>
       <c r="B60" s="4">
         <f t="shared" si="0"/>
         <v>56</v>
       </c>
-      <c r="C60" s="1" t="s">
+      <c r="C60" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D60" s="6">
@@ -4026,14 +4058,14 @@
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" s="5">
+      <c r="A61" s="54">
         <v>2024</v>
       </c>
       <c r="B61" s="4">
         <f t="shared" si="0"/>
         <v>57</v>
       </c>
-      <c r="C61" s="1" t="s">
+      <c r="C61" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D61" s="6">
@@ -4044,14 +4076,14 @@
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" s="5">
+      <c r="A62" s="54">
         <v>2024</v>
       </c>
       <c r="B62" s="4">
         <f t="shared" si="0"/>
         <v>58</v>
       </c>
-      <c r="C62" s="1" t="s">
+      <c r="C62" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D62" s="6">
@@ -4062,14 +4094,14 @@
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" s="5">
+      <c r="A63" s="54">
         <v>2024</v>
       </c>
       <c r="B63" s="4">
         <f t="shared" si="0"/>
         <v>59</v>
       </c>
-      <c r="C63" s="1" t="s">
+      <c r="C63" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D63" s="6">
@@ -4080,14 +4112,14 @@
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" s="5">
+      <c r="A64" s="54">
         <v>2024</v>
       </c>
       <c r="B64" s="4">
         <f t="shared" si="0"/>
         <v>60</v>
       </c>
-      <c r="C64" s="1" t="s">
+      <c r="C64" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D64" s="6">
@@ -4098,14 +4130,14 @@
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A65" s="5">
+      <c r="A65" s="54">
         <v>2024</v>
       </c>
       <c r="B65" s="32">
         <f t="shared" si="0"/>
         <v>61</v>
       </c>
-      <c r="C65" s="33" t="s">
+      <c r="C65" s="55" t="s">
         <v>6</v>
       </c>
       <c r="D65" s="38">
@@ -4116,998 +4148,998 @@
       </c>
     </row>
     <row r="66" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A66" s="13"/>
-      <c r="B66" s="25">
+      <c r="A66" s="56"/>
+      <c r="B66" s="4">
         <v>62</v>
       </c>
-      <c r="C66" s="26" t="s">
+      <c r="C66" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D66" s="39">
+      <c r="D66" s="57">
         <v>241191101014</v>
       </c>
-      <c r="E66" s="40" t="s">
+      <c r="E66" s="58" t="s">
         <v>223</v>
       </c>
-      <c r="F66" s="31" t="s">
+      <c r="F66" s="59" t="s">
         <v>225</v>
       </c>
     </row>
     <row r="67" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="13"/>
-      <c r="B67" s="25">
+      <c r="A67" s="56"/>
+      <c r="B67" s="4">
         <v>63</v>
       </c>
-      <c r="C67" s="26" t="s">
+      <c r="C67" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D67" s="39">
+      <c r="D67" s="57">
         <v>241191101053</v>
       </c>
-      <c r="E67" s="40" t="s">
+      <c r="E67" s="58" t="s">
         <v>224</v>
       </c>
-      <c r="F67" s="31" t="s">
+      <c r="F67" s="59" t="s">
         <v>225</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A68" s="13"/>
-      <c r="B68" s="43">
+      <c r="A68" s="56"/>
+      <c r="B68" s="60">
         <v>64</v>
       </c>
-      <c r="C68" s="43" t="s">
+      <c r="C68" s="60" t="s">
         <v>6</v>
       </c>
-      <c r="D68" s="44">
+      <c r="D68" s="61">
         <v>241191101044</v>
       </c>
-      <c r="E68" s="45" t="s">
+      <c r="E68" s="62" t="s">
         <v>228</v>
       </c>
-      <c r="F68" s="45" t="s">
+      <c r="F68" s="62" t="s">
         <v>229</v>
       </c>
     </row>
     <row r="69" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A69" s="13"/>
-      <c r="B69" s="25">
+      <c r="A69" s="56"/>
+      <c r="B69" s="4">
         <v>65</v>
       </c>
-      <c r="C69" s="46" t="s">
+      <c r="C69" s="63" t="s">
         <v>6</v>
       </c>
-      <c r="D69" s="47">
+      <c r="D69" s="64">
         <v>241191101060</v>
       </c>
-      <c r="E69" s="48" t="s">
+      <c r="E69" s="65" t="s">
         <v>230</v>
       </c>
-      <c r="F69" s="31" t="s">
+      <c r="F69" s="59" t="s">
         <v>231</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A70" s="13"/>
+      <c r="A70" s="56"/>
       <c r="B70" s="14"/>
-      <c r="C70" s="15"/>
+      <c r="C70" s="16"/>
       <c r="D70" s="17"/>
       <c r="E70" s="18"/>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A71" s="13"/>
+      <c r="A71" s="56"/>
       <c r="B71" s="14"/>
-      <c r="C71" s="15"/>
+      <c r="C71" s="16"/>
       <c r="D71" s="17"/>
       <c r="E71" s="18"/>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A72" s="13"/>
+      <c r="A72" s="56"/>
       <c r="B72" s="14"/>
-      <c r="C72" s="15"/>
+      <c r="C72" s="16"/>
       <c r="D72" s="17"/>
       <c r="E72" s="18"/>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A73" s="13"/>
+      <c r="A73" s="56"/>
       <c r="B73" s="14"/>
-      <c r="C73" s="15"/>
+      <c r="C73" s="16"/>
       <c r="D73" s="17"/>
       <c r="E73" s="18"/>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A74" s="13"/>
+      <c r="A74" s="56"/>
       <c r="B74" s="14"/>
-      <c r="C74" s="15"/>
+      <c r="C74" s="16"/>
       <c r="D74" s="17"/>
       <c r="E74" s="18"/>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A75" s="13"/>
+      <c r="A75" s="56"/>
       <c r="B75" s="14"/>
-      <c r="C75" s="15"/>
+      <c r="C75" s="16"/>
       <c r="D75" s="17"/>
       <c r="E75" s="18"/>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A76" s="13"/>
+      <c r="A76" s="56"/>
       <c r="B76" s="14"/>
-      <c r="C76" s="15"/>
+      <c r="C76" s="16"/>
       <c r="D76" s="17"/>
       <c r="E76" s="18"/>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A77" s="13"/>
+      <c r="A77" s="56"/>
       <c r="B77" s="14"/>
-      <c r="C77" s="15"/>
+      <c r="C77" s="16"/>
       <c r="D77" s="17"/>
       <c r="E77" s="18"/>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A78" s="13"/>
+      <c r="A78" s="56"/>
       <c r="B78" s="14"/>
-      <c r="C78" s="15"/>
+      <c r="C78" s="16"/>
       <c r="D78" s="17"/>
       <c r="E78" s="18"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A79" s="13"/>
+      <c r="A79" s="56"/>
       <c r="B79" s="14"/>
-      <c r="C79" s="15"/>
+      <c r="C79" s="16"/>
       <c r="D79" s="17"/>
       <c r="E79" s="18"/>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A80" s="13"/>
+      <c r="A80" s="56"/>
       <c r="B80" s="14"/>
-      <c r="C80" s="15"/>
+      <c r="C80" s="16"/>
       <c r="D80" s="17"/>
       <c r="E80" s="18"/>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A81" s="13"/>
+      <c r="A81" s="56"/>
       <c r="B81" s="14"/>
-      <c r="C81" s="15"/>
+      <c r="C81" s="16"/>
       <c r="D81" s="17"/>
       <c r="E81" s="18"/>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A82" s="13"/>
+      <c r="A82" s="56"/>
       <c r="B82" s="14"/>
-      <c r="C82" s="15"/>
+      <c r="C82" s="16"/>
       <c r="D82" s="17"/>
       <c r="E82" s="18"/>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A83" s="13"/>
+      <c r="A83" s="56"/>
       <c r="B83" s="14"/>
-      <c r="C83" s="15"/>
+      <c r="C83" s="16"/>
       <c r="D83" s="17"/>
       <c r="E83" s="18"/>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A84" s="13"/>
+      <c r="A84" s="56"/>
       <c r="B84" s="14"/>
-      <c r="C84" s="15"/>
+      <c r="C84" s="16"/>
       <c r="D84" s="17"/>
       <c r="E84" s="18"/>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A85" s="13"/>
+      <c r="A85" s="56"/>
       <c r="B85" s="14"/>
-      <c r="C85" s="15"/>
+      <c r="C85" s="16"/>
       <c r="D85" s="17"/>
       <c r="E85" s="18"/>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A86" s="13"/>
+      <c r="A86" s="56"/>
       <c r="B86" s="14"/>
-      <c r="C86" s="15"/>
+      <c r="C86" s="16"/>
       <c r="D86" s="17"/>
       <c r="E86" s="18"/>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A87" s="13"/>
+      <c r="A87" s="56"/>
       <c r="B87" s="14"/>
-      <c r="C87" s="15"/>
+      <c r="C87" s="16"/>
       <c r="D87" s="17"/>
       <c r="E87" s="18"/>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A88" s="13"/>
+      <c r="A88" s="56"/>
       <c r="B88" s="14"/>
-      <c r="C88" s="15"/>
+      <c r="C88" s="16"/>
       <c r="D88" s="17"/>
       <c r="E88" s="18"/>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A89" s="13"/>
+      <c r="A89" s="56"/>
       <c r="B89" s="14"/>
-      <c r="C89" s="15"/>
+      <c r="C89" s="16"/>
       <c r="D89" s="17"/>
       <c r="E89" s="18"/>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A90" s="13"/>
+      <c r="A90" s="56"/>
       <c r="B90" s="14"/>
-      <c r="C90" s="15"/>
+      <c r="C90" s="16"/>
       <c r="D90" s="17"/>
       <c r="E90" s="18"/>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A91" s="13"/>
+      <c r="A91" s="56"/>
       <c r="B91" s="14"/>
-      <c r="C91" s="15"/>
+      <c r="C91" s="16"/>
       <c r="D91" s="17"/>
       <c r="E91" s="18"/>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A92" s="13"/>
+      <c r="A92" s="56"/>
       <c r="B92" s="14"/>
-      <c r="C92" s="15"/>
+      <c r="C92" s="16"/>
       <c r="D92" s="17"/>
       <c r="E92" s="18"/>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A93" s="13"/>
+      <c r="A93" s="56"/>
       <c r="B93" s="14"/>
-      <c r="C93" s="15"/>
+      <c r="C93" s="16"/>
       <c r="D93" s="17"/>
       <c r="E93" s="18"/>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A94" s="13"/>
+      <c r="A94" s="56"/>
       <c r="B94" s="14"/>
-      <c r="C94" s="15"/>
+      <c r="C94" s="16"/>
       <c r="D94" s="17"/>
       <c r="E94" s="18"/>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A95" s="13"/>
+      <c r="A95" s="56"/>
       <c r="B95" s="14"/>
-      <c r="C95" s="15"/>
+      <c r="C95" s="16"/>
       <c r="D95" s="17"/>
       <c r="E95" s="18"/>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A96" s="13"/>
+      <c r="A96" s="56"/>
       <c r="B96" s="14"/>
-      <c r="C96" s="15"/>
+      <c r="C96" s="16"/>
       <c r="D96" s="17"/>
       <c r="E96" s="18"/>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A97" s="13"/>
+      <c r="A97" s="56"/>
       <c r="B97" s="14"/>
-      <c r="C97" s="15"/>
+      <c r="C97" s="16"/>
       <c r="D97" s="17"/>
       <c r="E97" s="18"/>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A98" s="13"/>
+      <c r="A98" s="56"/>
       <c r="B98" s="14"/>
-      <c r="C98" s="15"/>
+      <c r="C98" s="16"/>
       <c r="D98" s="17"/>
       <c r="E98" s="18"/>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A99" s="13"/>
+      <c r="A99" s="56"/>
       <c r="B99" s="14"/>
-      <c r="C99" s="15"/>
+      <c r="C99" s="16"/>
       <c r="D99" s="17"/>
       <c r="E99" s="18"/>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A100" s="13"/>
+      <c r="A100" s="56"/>
       <c r="B100" s="14"/>
-      <c r="C100" s="15"/>
+      <c r="C100" s="16"/>
       <c r="D100" s="17"/>
       <c r="E100" s="18"/>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A101" s="13"/>
+      <c r="A101" s="56"/>
       <c r="B101" s="14"/>
-      <c r="C101" s="15"/>
+      <c r="C101" s="16"/>
       <c r="D101" s="17"/>
       <c r="E101" s="18"/>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A102" s="13"/>
+      <c r="A102" s="56"/>
       <c r="B102" s="14"/>
-      <c r="C102" s="15"/>
+      <c r="C102" s="16"/>
       <c r="D102" s="17"/>
       <c r="E102" s="18"/>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A103" s="13"/>
+      <c r="A103" s="56"/>
       <c r="B103" s="14"/>
-      <c r="C103" s="15"/>
+      <c r="C103" s="16"/>
       <c r="D103" s="17"/>
       <c r="E103" s="18"/>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A104" s="13"/>
+      <c r="A104" s="56"/>
       <c r="B104" s="14"/>
-      <c r="C104" s="15"/>
+      <c r="C104" s="16"/>
       <c r="D104" s="17"/>
       <c r="E104" s="18"/>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A105" s="13"/>
+      <c r="A105" s="56"/>
       <c r="B105" s="14"/>
-      <c r="C105" s="15"/>
+      <c r="C105" s="16"/>
       <c r="D105" s="17"/>
       <c r="E105" s="18"/>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A106" s="13"/>
+      <c r="A106" s="56"/>
       <c r="B106" s="14"/>
-      <c r="C106" s="15"/>
+      <c r="C106" s="16"/>
       <c r="D106" s="17"/>
       <c r="E106" s="18"/>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A107" s="13"/>
+      <c r="A107" s="56"/>
       <c r="B107" s="14"/>
-      <c r="C107" s="15"/>
+      <c r="C107" s="16"/>
       <c r="D107" s="17"/>
       <c r="E107" s="19"/>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A108" s="13"/>
+      <c r="A108" s="56"/>
       <c r="B108" s="14"/>
-      <c r="C108" s="15"/>
+      <c r="C108" s="16"/>
       <c r="D108" s="17"/>
       <c r="E108" s="18"/>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A109" s="13"/>
+      <c r="A109" s="56"/>
       <c r="B109" s="14"/>
-      <c r="C109" s="15"/>
+      <c r="C109" s="16"/>
       <c r="D109" s="17"/>
       <c r="E109" s="18"/>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A110" s="13"/>
+      <c r="A110" s="56"/>
       <c r="B110" s="14"/>
-      <c r="C110" s="15"/>
+      <c r="C110" s="16"/>
       <c r="D110" s="17"/>
       <c r="E110" s="18"/>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A111" s="13"/>
+      <c r="A111" s="56"/>
       <c r="B111" s="14"/>
-      <c r="C111" s="15"/>
+      <c r="C111" s="16"/>
       <c r="D111" s="17"/>
       <c r="E111" s="18"/>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A112" s="13"/>
+      <c r="A112" s="56"/>
       <c r="B112" s="14"/>
-      <c r="C112" s="15"/>
+      <c r="C112" s="16"/>
       <c r="D112" s="17"/>
       <c r="E112" s="18"/>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A113" s="13"/>
+      <c r="A113" s="56"/>
       <c r="B113" s="14"/>
-      <c r="C113" s="15"/>
+      <c r="C113" s="16"/>
       <c r="D113" s="17"/>
       <c r="E113" s="18"/>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A114" s="13"/>
+      <c r="A114" s="56"/>
       <c r="B114" s="14"/>
-      <c r="C114" s="15"/>
+      <c r="C114" s="16"/>
       <c r="D114" s="17"/>
       <c r="E114" s="18"/>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A115" s="13"/>
+      <c r="A115" s="56"/>
       <c r="B115" s="14"/>
-      <c r="C115" s="15"/>
+      <c r="C115" s="16"/>
       <c r="D115" s="17"/>
       <c r="E115" s="18"/>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A116" s="13"/>
+      <c r="A116" s="56"/>
       <c r="B116" s="14"/>
-      <c r="C116" s="15"/>
+      <c r="C116" s="16"/>
       <c r="D116" s="17"/>
       <c r="E116" s="18"/>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A117" s="13"/>
+      <c r="A117" s="56"/>
       <c r="B117" s="14"/>
-      <c r="C117" s="15"/>
+      <c r="C117" s="16"/>
       <c r="D117" s="17"/>
       <c r="E117" s="18"/>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A118" s="13"/>
+      <c r="A118" s="56"/>
       <c r="B118" s="14"/>
-      <c r="C118" s="15"/>
+      <c r="C118" s="16"/>
       <c r="D118" s="17"/>
       <c r="E118" s="18"/>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A119" s="13"/>
+      <c r="A119" s="56"/>
       <c r="B119" s="14"/>
-      <c r="C119" s="15"/>
+      <c r="C119" s="16"/>
       <c r="D119" s="17"/>
       <c r="E119" s="18"/>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A120" s="13"/>
+      <c r="A120" s="56"/>
       <c r="B120" s="14"/>
-      <c r="C120" s="15"/>
+      <c r="C120" s="16"/>
       <c r="D120" s="17"/>
       <c r="E120" s="18"/>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A121" s="13"/>
+      <c r="A121" s="56"/>
       <c r="B121" s="14"/>
-      <c r="C121" s="15"/>
+      <c r="C121" s="16"/>
       <c r="D121" s="17"/>
       <c r="E121" s="18"/>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A122" s="13"/>
+      <c r="A122" s="56"/>
       <c r="B122" s="14"/>
-      <c r="C122" s="15"/>
+      <c r="C122" s="16"/>
       <c r="D122" s="17"/>
       <c r="E122" s="18"/>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A123" s="13"/>
+      <c r="A123" s="56"/>
       <c r="B123" s="14"/>
-      <c r="C123" s="15"/>
+      <c r="C123" s="16"/>
       <c r="D123" s="17"/>
       <c r="E123" s="18"/>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A124" s="13"/>
+      <c r="A124" s="56"/>
       <c r="B124" s="14"/>
-      <c r="C124" s="15"/>
+      <c r="C124" s="16"/>
       <c r="D124" s="17"/>
       <c r="E124" s="18"/>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A125" s="13"/>
+      <c r="A125" s="56"/>
       <c r="B125" s="14"/>
-      <c r="C125" s="15"/>
+      <c r="C125" s="16"/>
       <c r="D125" s="17"/>
       <c r="E125" s="18"/>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A126" s="13"/>
+      <c r="A126" s="56"/>
       <c r="B126" s="14"/>
-      <c r="C126" s="15"/>
+      <c r="C126" s="16"/>
       <c r="D126" s="17"/>
       <c r="E126" s="18"/>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A127" s="13"/>
+      <c r="A127" s="56"/>
       <c r="B127" s="14"/>
-      <c r="C127" s="15"/>
+      <c r="C127" s="16"/>
       <c r="D127" s="17"/>
       <c r="E127" s="18"/>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A128" s="13"/>
+      <c r="A128" s="56"/>
       <c r="B128" s="14"/>
-      <c r="C128" s="15"/>
+      <c r="C128" s="16"/>
       <c r="D128" s="17"/>
       <c r="E128" s="18"/>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A129" s="13"/>
+      <c r="A129" s="56"/>
       <c r="B129" s="14"/>
-      <c r="C129" s="15"/>
+      <c r="C129" s="16"/>
       <c r="D129" s="16"/>
       <c r="E129" s="16"/>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A130" s="13"/>
+      <c r="A130" s="56"/>
       <c r="B130" s="14"/>
-      <c r="C130" s="15"/>
+      <c r="C130" s="16"/>
       <c r="D130" s="17"/>
       <c r="E130" s="20"/>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A131" s="13"/>
+      <c r="A131" s="56"/>
       <c r="B131" s="14"/>
-      <c r="C131" s="15"/>
+      <c r="C131" s="16"/>
       <c r="D131" s="17"/>
       <c r="E131" s="20"/>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A132" s="13"/>
+      <c r="A132" s="56"/>
       <c r="B132" s="14"/>
-      <c r="C132" s="15"/>
+      <c r="C132" s="16"/>
       <c r="D132" s="17"/>
       <c r="E132" s="20"/>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A133" s="13"/>
+      <c r="A133" s="56"/>
       <c r="B133" s="14"/>
-      <c r="C133" s="15"/>
+      <c r="C133" s="16"/>
       <c r="D133" s="17"/>
       <c r="E133" s="20"/>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A134" s="13"/>
+      <c r="A134" s="56"/>
       <c r="B134" s="14"/>
-      <c r="C134" s="15"/>
+      <c r="C134" s="16"/>
       <c r="D134" s="17"/>
       <c r="E134" s="20"/>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A135" s="13"/>
+      <c r="A135" s="56"/>
       <c r="B135" s="14"/>
-      <c r="C135" s="15"/>
+      <c r="C135" s="16"/>
       <c r="D135" s="17"/>
       <c r="E135" s="20"/>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A136" s="13"/>
+      <c r="A136" s="56"/>
       <c r="B136" s="14"/>
-      <c r="C136" s="15"/>
+      <c r="C136" s="16"/>
       <c r="D136" s="17"/>
       <c r="E136" s="20"/>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A137" s="13"/>
+      <c r="A137" s="56"/>
       <c r="B137" s="14"/>
-      <c r="C137" s="15"/>
+      <c r="C137" s="16"/>
       <c r="D137" s="17"/>
       <c r="E137" s="20"/>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A138" s="13"/>
+      <c r="A138" s="56"/>
       <c r="B138" s="14"/>
-      <c r="C138" s="15"/>
+      <c r="C138" s="16"/>
       <c r="D138" s="17"/>
       <c r="E138" s="20"/>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A139" s="13"/>
+      <c r="A139" s="56"/>
       <c r="B139" s="14"/>
-      <c r="C139" s="15"/>
+      <c r="C139" s="16"/>
       <c r="D139" s="17"/>
       <c r="E139" s="20"/>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A140" s="13"/>
+      <c r="A140" s="56"/>
       <c r="B140" s="14"/>
-      <c r="C140" s="15"/>
+      <c r="C140" s="16"/>
       <c r="D140" s="17"/>
       <c r="E140" s="20"/>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A141" s="13"/>
+      <c r="A141" s="56"/>
       <c r="B141" s="14"/>
-      <c r="C141" s="15"/>
+      <c r="C141" s="16"/>
       <c r="D141" s="17"/>
       <c r="E141" s="20"/>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A142" s="13"/>
+      <c r="A142" s="56"/>
       <c r="B142" s="14"/>
-      <c r="C142" s="15"/>
+      <c r="C142" s="16"/>
       <c r="D142" s="17"/>
       <c r="E142" s="20"/>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A143" s="13"/>
+      <c r="A143" s="56"/>
       <c r="B143" s="14"/>
-      <c r="C143" s="15"/>
+      <c r="C143" s="16"/>
       <c r="D143" s="17"/>
       <c r="E143" s="20"/>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A144" s="13"/>
+      <c r="A144" s="56"/>
       <c r="B144" s="14"/>
-      <c r="C144" s="15"/>
+      <c r="C144" s="16"/>
       <c r="D144" s="17"/>
       <c r="E144" s="20"/>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A145" s="13"/>
+      <c r="A145" s="56"/>
       <c r="B145" s="14"/>
-      <c r="C145" s="15"/>
+      <c r="C145" s="16"/>
       <c r="D145" s="17"/>
       <c r="E145" s="20"/>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A146" s="13"/>
+      <c r="A146" s="56"/>
       <c r="B146" s="14"/>
-      <c r="C146" s="15"/>
+      <c r="C146" s="16"/>
       <c r="D146" s="17"/>
       <c r="E146" s="20"/>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A147" s="13"/>
+      <c r="A147" s="56"/>
       <c r="B147" s="14"/>
-      <c r="C147" s="15"/>
+      <c r="C147" s="16"/>
       <c r="D147" s="17"/>
       <c r="E147" s="20"/>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A148" s="13"/>
+      <c r="A148" s="56"/>
       <c r="B148" s="14"/>
-      <c r="C148" s="15"/>
+      <c r="C148" s="16"/>
       <c r="D148" s="17"/>
       <c r="E148" s="20"/>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A149" s="13"/>
+      <c r="A149" s="56"/>
       <c r="B149" s="14"/>
-      <c r="C149" s="15"/>
+      <c r="C149" s="16"/>
       <c r="D149" s="17"/>
       <c r="E149" s="20"/>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A150" s="13"/>
+      <c r="A150" s="56"/>
       <c r="B150" s="14"/>
-      <c r="C150" s="15"/>
+      <c r="C150" s="16"/>
       <c r="D150" s="17"/>
       <c r="E150" s="20"/>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A151" s="13"/>
+      <c r="A151" s="56"/>
       <c r="B151" s="14"/>
-      <c r="C151" s="15"/>
+      <c r="C151" s="16"/>
       <c r="D151" s="17"/>
       <c r="E151" s="20"/>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A152" s="13"/>
+      <c r="A152" s="56"/>
       <c r="B152" s="14"/>
-      <c r="C152" s="15"/>
+      <c r="C152" s="16"/>
       <c r="D152" s="17"/>
       <c r="E152" s="20"/>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A153" s="13"/>
+      <c r="A153" s="56"/>
       <c r="B153" s="14"/>
-      <c r="C153" s="15"/>
+      <c r="C153" s="16"/>
       <c r="D153" s="17"/>
       <c r="E153" s="20"/>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A154" s="13"/>
+      <c r="A154" s="56"/>
       <c r="B154" s="14"/>
-      <c r="C154" s="15"/>
+      <c r="C154" s="16"/>
       <c r="D154" s="17"/>
       <c r="E154" s="20"/>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A155" s="13"/>
+      <c r="A155" s="56"/>
       <c r="B155" s="14"/>
-      <c r="C155" s="15"/>
+      <c r="C155" s="16"/>
       <c r="D155" s="17"/>
       <c r="E155" s="20"/>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A156" s="13"/>
+      <c r="A156" s="56"/>
       <c r="B156" s="14"/>
-      <c r="C156" s="15"/>
+      <c r="C156" s="16"/>
       <c r="D156" s="17"/>
       <c r="E156" s="20"/>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A157" s="13"/>
+      <c r="A157" s="56"/>
       <c r="B157" s="14"/>
-      <c r="C157" s="15"/>
+      <c r="C157" s="16"/>
       <c r="D157" s="17"/>
       <c r="E157" s="20"/>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A158" s="13"/>
+      <c r="A158" s="56"/>
       <c r="B158" s="14"/>
-      <c r="C158" s="15"/>
+      <c r="C158" s="16"/>
       <c r="D158" s="17"/>
       <c r="E158" s="20"/>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A159" s="13"/>
+      <c r="A159" s="56"/>
       <c r="B159" s="14"/>
-      <c r="C159" s="15"/>
+      <c r="C159" s="16"/>
       <c r="D159" s="17"/>
       <c r="E159" s="20"/>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A160" s="13"/>
+      <c r="A160" s="56"/>
       <c r="B160" s="14"/>
-      <c r="C160" s="15"/>
+      <c r="C160" s="16"/>
       <c r="D160" s="17"/>
       <c r="E160" s="20"/>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A161" s="13"/>
+      <c r="A161" s="56"/>
       <c r="B161" s="14"/>
-      <c r="C161" s="15"/>
+      <c r="C161" s="16"/>
       <c r="D161" s="17"/>
       <c r="E161" s="20"/>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A162" s="13"/>
+      <c r="A162" s="56"/>
       <c r="B162" s="14"/>
-      <c r="C162" s="15"/>
+      <c r="C162" s="16"/>
       <c r="D162" s="17"/>
       <c r="E162" s="20"/>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A163" s="13"/>
+      <c r="A163" s="56"/>
       <c r="B163" s="14"/>
-      <c r="C163" s="15"/>
+      <c r="C163" s="16"/>
       <c r="D163" s="21"/>
       <c r="E163" s="18"/>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A164" s="13"/>
+      <c r="A164" s="56"/>
       <c r="B164" s="14"/>
-      <c r="C164" s="15"/>
+      <c r="C164" s="16"/>
       <c r="D164" s="21"/>
       <c r="E164" s="18"/>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A165" s="13"/>
+      <c r="A165" s="56"/>
       <c r="B165" s="14"/>
-      <c r="C165" s="22"/>
+      <c r="C165" s="14"/>
       <c r="D165" s="16"/>
       <c r="E165" s="16"/>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A166" s="13"/>
+      <c r="A166" s="56"/>
       <c r="B166" s="14"/>
-      <c r="C166" s="22"/>
+      <c r="C166" s="14"/>
       <c r="D166" s="17"/>
       <c r="E166" s="20"/>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A167" s="13"/>
+      <c r="A167" s="56"/>
       <c r="B167" s="14"/>
-      <c r="C167" s="22"/>
+      <c r="C167" s="14"/>
       <c r="D167" s="17"/>
       <c r="E167" s="20"/>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A168" s="13"/>
+      <c r="A168" s="56"/>
       <c r="B168" s="14"/>
-      <c r="C168" s="22"/>
+      <c r="C168" s="14"/>
       <c r="D168" s="17"/>
       <c r="E168" s="20"/>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A169" s="13"/>
+      <c r="A169" s="56"/>
       <c r="B169" s="14"/>
-      <c r="C169" s="22"/>
+      <c r="C169" s="14"/>
       <c r="D169" s="17"/>
       <c r="E169" s="20"/>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A170" s="13"/>
+      <c r="A170" s="56"/>
       <c r="B170" s="14"/>
-      <c r="C170" s="22"/>
+      <c r="C170" s="14"/>
       <c r="D170" s="17"/>
       <c r="E170" s="20"/>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A171" s="13"/>
+      <c r="A171" s="56"/>
       <c r="B171" s="14"/>
-      <c r="C171" s="22"/>
+      <c r="C171" s="14"/>
       <c r="D171" s="17"/>
       <c r="E171" s="20"/>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A172" s="13"/>
+      <c r="A172" s="56"/>
       <c r="B172" s="14"/>
-      <c r="C172" s="22"/>
+      <c r="C172" s="14"/>
       <c r="D172" s="17"/>
       <c r="E172" s="20"/>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A173" s="13"/>
+      <c r="A173" s="56"/>
       <c r="B173" s="14"/>
-      <c r="C173" s="22"/>
+      <c r="C173" s="14"/>
       <c r="D173" s="17"/>
       <c r="E173" s="20"/>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A174" s="13"/>
+      <c r="A174" s="56"/>
       <c r="B174" s="14"/>
-      <c r="C174" s="22"/>
+      <c r="C174" s="14"/>
       <c r="D174" s="17"/>
       <c r="E174" s="20"/>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A175" s="13"/>
+      <c r="A175" s="56"/>
       <c r="B175" s="14"/>
-      <c r="C175" s="22"/>
+      <c r="C175" s="14"/>
       <c r="D175" s="17"/>
       <c r="E175" s="20"/>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A176" s="13"/>
+      <c r="A176" s="56"/>
       <c r="B176" s="14"/>
-      <c r="C176" s="22"/>
+      <c r="C176" s="14"/>
       <c r="D176" s="17"/>
       <c r="E176" s="20"/>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A177" s="13"/>
+      <c r="A177" s="56"/>
       <c r="B177" s="14"/>
-      <c r="C177" s="22"/>
+      <c r="C177" s="14"/>
       <c r="D177" s="17"/>
       <c r="E177" s="20"/>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A178" s="13"/>
+      <c r="A178" s="56"/>
       <c r="B178" s="14"/>
-      <c r="C178" s="22"/>
+      <c r="C178" s="14"/>
       <c r="D178" s="17"/>
       <c r="E178" s="20"/>
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A179" s="13"/>
+      <c r="A179" s="56"/>
       <c r="B179" s="14"/>
-      <c r="C179" s="22"/>
+      <c r="C179" s="14"/>
       <c r="D179" s="17"/>
       <c r="E179" s="20"/>
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A180" s="13"/>
+      <c r="A180" s="56"/>
       <c r="B180" s="14"/>
-      <c r="C180" s="22"/>
+      <c r="C180" s="14"/>
       <c r="D180" s="17"/>
       <c r="E180" s="20"/>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A181" s="13"/>
+      <c r="A181" s="56"/>
       <c r="B181" s="14"/>
-      <c r="C181" s="22"/>
+      <c r="C181" s="14"/>
       <c r="D181" s="17"/>
       <c r="E181" s="20"/>
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A182" s="13"/>
+      <c r="A182" s="56"/>
       <c r="B182" s="14"/>
-      <c r="C182" s="22"/>
+      <c r="C182" s="14"/>
       <c r="D182" s="17"/>
       <c r="E182" s="20"/>
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A183" s="13"/>
+      <c r="A183" s="56"/>
       <c r="B183" s="14"/>
-      <c r="C183" s="22"/>
+      <c r="C183" s="14"/>
       <c r="D183" s="17"/>
       <c r="E183" s="20"/>
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A184" s="13"/>
+      <c r="A184" s="56"/>
       <c r="B184" s="14"/>
-      <c r="C184" s="22"/>
+      <c r="C184" s="14"/>
       <c r="D184" s="17"/>
       <c r="E184" s="20"/>
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A185" s="13"/>
+      <c r="A185" s="56"/>
       <c r="B185" s="14"/>
-      <c r="C185" s="22"/>
+      <c r="C185" s="14"/>
       <c r="D185" s="17"/>
       <c r="E185" s="20"/>
     </row>
     <row r="186" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A186" s="13"/>
+      <c r="A186" s="56"/>
       <c r="B186" s="14"/>
-      <c r="C186" s="22"/>
+      <c r="C186" s="14"/>
       <c r="D186" s="17"/>
       <c r="E186" s="20"/>
     </row>
     <row r="187" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A187" s="13"/>
+      <c r="A187" s="56"/>
       <c r="B187" s="14"/>
-      <c r="C187" s="22"/>
+      <c r="C187" s="14"/>
       <c r="D187" s="17"/>
       <c r="E187" s="20"/>
     </row>
     <row r="188" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A188" s="13"/>
+      <c r="A188" s="56"/>
       <c r="B188" s="14"/>
-      <c r="C188" s="22"/>
+      <c r="C188" s="14"/>
       <c r="D188" s="17"/>
       <c r="E188" s="20"/>
     </row>
     <row r="189" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A189" s="13"/>
+      <c r="A189" s="56"/>
       <c r="B189" s="14"/>
-      <c r="C189" s="22"/>
+      <c r="C189" s="14"/>
       <c r="D189" s="17"/>
       <c r="E189" s="20"/>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A190" s="13"/>
+      <c r="A190" s="56"/>
       <c r="B190" s="14"/>
-      <c r="C190" s="22"/>
+      <c r="C190" s="14"/>
       <c r="D190" s="17"/>
       <c r="E190" s="20"/>
     </row>
     <row r="191" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A191" s="13"/>
+      <c r="A191" s="56"/>
       <c r="B191" s="14"/>
-      <c r="C191" s="22"/>
+      <c r="C191" s="14"/>
       <c r="D191" s="17"/>
       <c r="E191" s="20"/>
     </row>
     <row r="192" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A192" s="13"/>
+      <c r="A192" s="56"/>
       <c r="B192" s="14"/>
-      <c r="C192" s="22"/>
+      <c r="C192" s="14"/>
       <c r="D192" s="17"/>
       <c r="E192" s="20"/>
     </row>
     <row r="193" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A193" s="13"/>
+      <c r="A193" s="56"/>
       <c r="B193" s="14"/>
-      <c r="C193" s="22"/>
+      <c r="C193" s="14"/>
       <c r="D193" s="17"/>
       <c r="E193" s="20"/>
     </row>
     <row r="194" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A194" s="13"/>
+      <c r="A194" s="56"/>
       <c r="B194" s="14"/>
-      <c r="C194" s="22"/>
+      <c r="C194" s="14"/>
       <c r="D194" s="17"/>
       <c r="E194" s="20"/>
     </row>
     <row r="195" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A195" s="13"/>
+      <c r="A195" s="56"/>
       <c r="B195" s="14"/>
-      <c r="C195" s="22"/>
+      <c r="C195" s="14"/>
       <c r="D195" s="17"/>
       <c r="E195" s="20"/>
     </row>
     <row r="196" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A196" s="13"/>
+      <c r="A196" s="56"/>
       <c r="B196" s="14"/>
-      <c r="C196" s="22"/>
+      <c r="C196" s="14"/>
       <c r="D196" s="17"/>
       <c r="E196" s="20"/>
     </row>
     <row r="197" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A197" s="13"/>
+      <c r="A197" s="56"/>
       <c r="B197" s="14"/>
-      <c r="C197" s="22"/>
+      <c r="C197" s="14"/>
       <c r="D197" s="17"/>
       <c r="E197" s="20"/>
     </row>
     <row r="198" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A198" s="13"/>
+      <c r="A198" s="56"/>
       <c r="B198" s="14"/>
-      <c r="C198" s="22"/>
+      <c r="C198" s="14"/>
       <c r="D198" s="17"/>
       <c r="E198" s="20"/>
     </row>
     <row r="199" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A199" s="13"/>
+      <c r="A199" s="56"/>
       <c r="B199" s="14"/>
-      <c r="C199" s="22"/>
+      <c r="C199" s="14"/>
       <c r="D199" s="17"/>
       <c r="E199" s="20"/>
     </row>
     <row r="200" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A200" s="13"/>
+      <c r="A200" s="56"/>
       <c r="B200" s="14"/>
-      <c r="C200" s="22"/>
+      <c r="C200" s="14"/>
       <c r="D200" s="17"/>
       <c r="E200" s="20"/>
     </row>
     <row r="201" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A201" s="13"/>
+      <c r="A201" s="56"/>
       <c r="B201" s="14"/>
-      <c r="C201" s="22"/>
+      <c r="C201" s="14"/>
       <c r="D201" s="17"/>
       <c r="E201" s="20"/>
     </row>
@@ -5188,11 +5220,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="52"/>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
+      <c r="A1" s="46"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
     </row>
     <row r="2" spans="1:5" s="24" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="23"/>
@@ -5206,13 +5238,13 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="53" t="s">
+      <c r="A3" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
-      <c r="D3" s="53"/>
-      <c r="E3" s="53"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -6970,11 +7002,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="52"/>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
+      <c r="A1" s="46"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
     </row>
     <row r="2" spans="1:5" s="24" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="23"/>
@@ -6988,13 +7020,13 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="54" t="s">
+      <c r="A3" s="47" t="s">
         <v>206</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
-      <c r="D3" s="53"/>
-      <c r="E3" s="53"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -7961,7 +7993,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.42578125" hidden="1" customWidth="1"/>
@@ -7972,11 +8004,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="66" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="52"/>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
+      <c r="A1" s="46"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
     </row>
     <row r="2" spans="1:5" s="24" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="23"/>
@@ -7990,13 +8022,13 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="54" t="s">
+      <c r="A3" s="47" t="s">
         <v>206</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
-      <c r="D3" s="53"/>
-      <c r="E3" s="53"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -8518,7 +8550,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5">
         <v>2024</v>
       </c>
@@ -8536,7 +8568,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
         <v>2024</v>
       </c>
@@ -8554,7 +8586,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5">
         <v>2024</v>
       </c>
@@ -8572,7 +8604,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="5">
         <v>2024</v>
       </c>
@@ -8590,7 +8622,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="5">
         <v>2024</v>
       </c>
@@ -8608,7 +8640,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5">
         <v>2024</v>
       </c>
@@ -8626,7 +8658,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5">
         <v>2024</v>
       </c>
@@ -8643,8 +8675,11 @@
       <c r="E39" s="11" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N39" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="5">
         <v>2024</v>
       </c>
@@ -8658,19 +8693,19 @@
       <c r="D40" s="6">
         <v>241191101182</v>
       </c>
-      <c r="E40" s="51" t="s">
+      <c r="E40" s="45" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B41" s="49">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B41" s="43">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
       <c r="C41" s="25" t="s">
         <v>169</v>
       </c>
-      <c r="D41" s="50">
+      <c r="D41" s="44">
         <v>241191101203</v>
       </c>
       <c r="E41" s="28" t="s">

</xml_diff>